<commit_message>
fix: Move detail pages back to pages/, fix all broken links, 116/116 tests pass
- Moved 29 detail pages from pages/_detail/ back to pages/ (Streamlit
  doesn't support page_link to subdirectories)
- Fixed all pages/_detail/ references to pages/ across 8 files
- Fixed broken link: 13_Client_Presentation.py → 13_Document_Hub.py
- Added full_system_test.py — comprehensive 116-point test suite
- ALL tests pass: syntax (82), imports (11), links (0 broken),
  config (46/46), database (15 tables), calculations (21/21),
  documents (DOCX+PPTX+XLSX+PDF), drawings (162), APIs (3/3),
  self-healing (100%), agro (6 crops), presenter (15 slides + AI copilot)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/auto_synced/Financial_Model_30MT_Uttar_Pradesh.xlsx
+++ b/data/auto_synced/Financial_Model_30MT_Uttar_Pradesh.xlsx
@@ -574,7 +574,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Rs 1273 Lakhs</t>
+          <t>Rs 1232 Lakhs</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Rs 21.9 Lakhs</t>
+          <t>Rs 20.6 Lakhs</t>
         </is>
       </c>
     </row>
@@ -610,7 +610,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>21.9%</t>
+          <t>20.7%</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>34.3%</t>
+          <t>32.2%</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2.01x</t>
+          <t>1.93x</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>52 months</t>
+          <t>54 months</t>
         </is>
       </c>
     </row>
@@ -746,19 +746,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1488</v>
+        <v>1440</v>
       </c>
       <c r="D2" t="n">
-        <v>598.92</v>
+        <v>579.6</v>
       </c>
       <c r="E2" t="n">
-        <v>312.48</v>
+        <v>302.4</v>
       </c>
       <c r="F2" t="n">
         <v>55.8</v>
       </c>
       <c r="G2" t="n">
-        <v>230.64</v>
+        <v>221.4</v>
       </c>
       <c r="H2" t="n">
         <v>120</v>
@@ -767,19 +767,19 @@
         <v>82.8</v>
       </c>
       <c r="J2" t="n">
-        <v>27.84</v>
+        <v>18.6</v>
       </c>
       <c r="K2" t="n">
-        <v>6.96</v>
+        <v>4.65</v>
       </c>
       <c r="L2" t="n">
-        <v>20.88</v>
+        <v>13.95</v>
       </c>
       <c r="M2" t="n">
-        <v>140.88</v>
+        <v>133.95</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="3">
@@ -792,19 +792,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2046</v>
+        <v>1980</v>
       </c>
       <c r="D3" t="n">
-        <v>823.52</v>
+        <v>796.95</v>
       </c>
       <c r="E3" t="n">
-        <v>429.66</v>
+        <v>415.8</v>
       </c>
       <c r="F3" t="n">
         <v>55.8</v>
       </c>
       <c r="G3" t="n">
-        <v>338.06</v>
+        <v>325.35</v>
       </c>
       <c r="H3" t="n">
         <v>120</v>
@@ -813,19 +813,19 @@
         <v>82.8</v>
       </c>
       <c r="J3" t="n">
-        <v>135.25</v>
+        <v>122.55</v>
       </c>
       <c r="K3" t="n">
-        <v>33.81</v>
+        <v>30.64</v>
       </c>
       <c r="L3" t="n">
-        <v>101.44</v>
+        <v>91.91</v>
       </c>
       <c r="M3" t="n">
-        <v>221.44</v>
+        <v>211.91</v>
       </c>
       <c r="N3" t="n">
-        <v>1.47</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="4">
@@ -838,19 +838,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2604</v>
+        <v>2520</v>
       </c>
       <c r="D4" t="n">
-        <v>1048.11</v>
+        <v>1014.3</v>
       </c>
       <c r="E4" t="n">
-        <v>546.84</v>
+        <v>529.2</v>
       </c>
       <c r="F4" t="n">
         <v>55.8</v>
       </c>
       <c r="G4" t="n">
-        <v>445.47</v>
+        <v>429.3</v>
       </c>
       <c r="H4" t="n">
         <v>120</v>
@@ -859,19 +859,19 @@
         <v>82.8</v>
       </c>
       <c r="J4" t="n">
-        <v>242.67</v>
+        <v>226.5</v>
       </c>
       <c r="K4" t="n">
-        <v>60.67</v>
+        <v>56.62</v>
       </c>
       <c r="L4" t="n">
-        <v>182</v>
+        <v>169.87</v>
       </c>
       <c r="M4" t="n">
-        <v>302</v>
+        <v>289.87</v>
       </c>
       <c r="N4" t="n">
-        <v>2.01</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="5">
@@ -884,19 +884,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2976</v>
+        <v>2880</v>
       </c>
       <c r="D5" t="n">
-        <v>1197.84</v>
+        <v>1159.2</v>
       </c>
       <c r="E5" t="n">
-        <v>624.96</v>
+        <v>604.8</v>
       </c>
       <c r="F5" t="n">
         <v>55.8</v>
       </c>
       <c r="G5" t="n">
-        <v>517.08</v>
+        <v>498.6</v>
       </c>
       <c r="H5" t="n">
         <v>120</v>
@@ -905,19 +905,19 @@
         <v>82.8</v>
       </c>
       <c r="J5" t="n">
-        <v>314.28</v>
+        <v>295.8</v>
       </c>
       <c r="K5" t="n">
-        <v>78.56999999999999</v>
+        <v>73.95</v>
       </c>
       <c r="L5" t="n">
-        <v>235.71</v>
+        <v>221.85</v>
       </c>
       <c r="M5" t="n">
-        <v>355.71</v>
+        <v>341.85</v>
       </c>
       <c r="N5" t="n">
-        <v>2.37</v>
+        <v>2.28</v>
       </c>
     </row>
     <row r="6">
@@ -930,19 +930,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3162</v>
+        <v>3060</v>
       </c>
       <c r="D6" t="n">
-        <v>1272.7</v>
+        <v>1231.65</v>
       </c>
       <c r="E6" t="n">
-        <v>664.02</v>
+        <v>642.6</v>
       </c>
       <c r="F6" t="n">
         <v>55.8</v>
       </c>
       <c r="G6" t="n">
-        <v>552.88</v>
+        <v>533.25</v>
       </c>
       <c r="H6" t="n">
         <v>120</v>
@@ -951,19 +951,19 @@
         <v>82.8</v>
       </c>
       <c r="J6" t="n">
-        <v>350.08</v>
+        <v>330.45</v>
       </c>
       <c r="K6" t="n">
-        <v>87.52</v>
+        <v>82.61</v>
       </c>
       <c r="L6" t="n">
-        <v>262.56</v>
+        <v>247.84</v>
       </c>
       <c r="M6" t="n">
-        <v>382.56</v>
+        <v>367.84</v>
       </c>
       <c r="N6" t="n">
-        <v>2.55</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="7">
@@ -976,19 +976,19 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3348</v>
+        <v>3240</v>
       </c>
       <c r="D7" t="n">
-        <v>1347.57</v>
+        <v>1304.1</v>
       </c>
       <c r="E7" t="n">
-        <v>703.08</v>
+        <v>680.4</v>
       </c>
       <c r="F7" t="n">
         <v>55.8</v>
       </c>
       <c r="G7" t="n">
-        <v>588.6900000000001</v>
+        <v>567.9</v>
       </c>
       <c r="H7" t="n">
         <v>120</v>
@@ -997,19 +997,19 @@
         <v>82.8</v>
       </c>
       <c r="J7" t="n">
-        <v>385.89</v>
+        <v>365.1</v>
       </c>
       <c r="K7" t="n">
-        <v>96.47</v>
+        <v>91.27</v>
       </c>
       <c r="L7" t="n">
-        <v>289.42</v>
+        <v>273.82</v>
       </c>
       <c r="M7" t="n">
-        <v>409.42</v>
+        <v>393.82</v>
       </c>
       <c r="N7" t="n">
-        <v>2.73</v>
+        <v>2.62</v>
       </c>
     </row>
     <row r="8">
@@ -1022,19 +1022,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>3348</v>
+        <v>3240</v>
       </c>
       <c r="D8" t="n">
-        <v>1347.57</v>
+        <v>1304.1</v>
       </c>
       <c r="E8" t="n">
-        <v>703.08</v>
+        <v>680.4</v>
       </c>
       <c r="F8" t="n">
         <v>55.8</v>
       </c>
       <c r="G8" t="n">
-        <v>588.6900000000001</v>
+        <v>567.9</v>
       </c>
       <c r="H8" t="n">
         <v>120</v>
@@ -1043,19 +1043,19 @@
         <v>82.8</v>
       </c>
       <c r="J8" t="n">
-        <v>385.89</v>
+        <v>365.1</v>
       </c>
       <c r="K8" t="n">
-        <v>96.47</v>
+        <v>91.27</v>
       </c>
       <c r="L8" t="n">
-        <v>289.42</v>
+        <v>273.82</v>
       </c>
       <c r="M8" t="n">
-        <v>409.42</v>
+        <v>393.82</v>
       </c>
       <c r="N8" t="n">
-        <v>2.73</v>
+        <v>2.62</v>
       </c>
     </row>
   </sheetData>
@@ -1217,13 +1217,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>337.5</v>
+        <v>324.3</v>
       </c>
       <c r="C2" t="n">
-        <v>503.5</v>
+        <v>484.9</v>
       </c>
       <c r="D2" t="n">
-        <v>669.5</v>
+        <v>645.6</v>
       </c>
     </row>
     <row r="3">
@@ -1233,13 +1233,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>204.7</v>
+        <v>195.8</v>
       </c>
       <c r="C3" t="n">
-        <v>370.7</v>
+        <v>356.4</v>
       </c>
       <c r="D3" t="n">
-        <v>536.7</v>
+        <v>517.1</v>
       </c>
     </row>
     <row r="4">
@@ -1249,13 +1249,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>71.90000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="C4" t="n">
-        <v>237.9</v>
+        <v>227.9</v>
       </c>
       <c r="D4" t="n">
-        <v>403.9</v>
+        <v>388.5</v>
       </c>
     </row>
   </sheetData>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>300</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">

</xml_diff>